<commit_message>
Update application to v2 with advanced logging and rotating file handler
</commit_message>
<xml_diff>
--- a/Import Item Report 15-MAY-2026_01_34_PM.xlsx
+++ b/Import Item Report 15-MAY-2026_01_34_PM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\DOCS\SKODA Item Mismatch Checker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7E5103-85D9-4EB2-BAF5-853D11013EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{592EFB78-74BB-446B-8F31-C7DA6245D6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2394" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2393" uniqueCount="155">
   <si>
     <t>Job No</t>
   </si>
@@ -1385,8 +1385,8 @@
       <c r="J3" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>77</v>
+      <c r="K3" s="1">
+        <v>74089900</v>
       </c>
       <c r="L3" s="4">
         <v>1</v>

</xml_diff>